<commit_message>
docs: canonicalize tutorial workbook xml
</commit_message>
<xml_diff>
--- a/examples/data/tutorial_01_alphas.xlsx
+++ b/examples/data/tutorial_01_alphas.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
+    <workbookView activeTab="0" autoFilterDateGrouping="1" firstSheet="0" minimized="0" showHorizontalScroll="1" showSheetTabs="1" showVerticalScroll="1" tabRatio="600" visibility="visible"/>
   </bookViews>
   <sheets>
-    <sheet name="alphas" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="alphas" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -44,15 +44,15 @@
     </border>
   </borders>
   <cellStyleXfs count="1">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf borderId="0" fillId="0" fontId="0" numFmtId="0"/>
   </cellStyleXfs>
   <cellXfs count="1">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf borderId="0" fillId="0" fontId="0" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
+    <cellStyle builtinId="0" hidden="0" name="Normal" xfId="0"/>
   </cellStyles>
-  <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
+  <tableStyles count="0" defaultPivotStyle="PivotStyleLight16" defaultTableStyle="TableStyleMedium9"/>
   <colors>
     <indexedColors>
       <rgbColor rgb="00000000"/>
@@ -129,10 +129,10 @@
   <a:themeElements>
     <a:clrScheme name="Office">
       <a:dk1>
-        <a:sysClr val="windowText" lastClr="000000"/>
+        <a:sysClr lastClr="000000" val="windowText"/>
       </a:dk1>
       <a:lt1>
-        <a:sysClr val="window" lastClr="FFFFFF"/>
+        <a:sysClr lastClr="FFFFFF" val="window"/>
       </a:lt1>
       <a:dk2>
         <a:srgbClr val="1F497D"/>
@@ -288,7 +288,7 @@
         </a:gradFill>
       </a:fillStyleLst>
       <a:lnStyleLst>
-        <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:ln algn="ctr" cap="flat" cmpd="sng" w="9525">
           <a:solidFill>
             <a:schemeClr val="phClr">
               <a:shade val="95000"/>
@@ -297,13 +297,13 @@
           </a:solidFill>
           <a:prstDash val="solid"/>
         </a:ln>
-        <a:ln w="25400" cap="flat" cmpd="sng" algn="ctr">
+        <a:ln algn="ctr" cap="flat" cmpd="sng" w="25400">
           <a:solidFill>
             <a:schemeClr val="phClr"/>
           </a:solidFill>
           <a:prstDash val="solid"/>
         </a:ln>
-        <a:ln w="38100" cap="flat" cmpd="sng" algn="ctr">
+        <a:ln algn="ctr" cap="flat" cmpd="sng" w="38100">
           <a:solidFill>
             <a:schemeClr val="phClr"/>
           </a:solidFill>
@@ -313,7 +313,7 @@
       <a:effectStyleLst>
         <a:effectStyle>
           <a:effectLst>
-            <a:outerShdw blurRad="40000" dist="20000" dir="5400000" rotWithShape="0">
+            <a:outerShdw blurRad="40000" dir="5400000" dist="20000" rotWithShape="0">
               <a:srgbClr val="000000">
                 <a:alpha val="38000"/>
               </a:srgbClr>
@@ -322,7 +322,7 @@
         </a:effectStyle>
         <a:effectStyle>
           <a:effectLst>
-            <a:outerShdw blurRad="40000" dist="23000" dir="5400000" rotWithShape="0">
+            <a:outerShdw blurRad="40000" dir="5400000" dist="23000" rotWithShape="0">
               <a:srgbClr val="000000">
                 <a:alpha val="35000"/>
               </a:srgbClr>
@@ -331,7 +331,7 @@
         </a:effectStyle>
         <a:effectStyle>
           <a:effectLst>
-            <a:outerShdw blurRad="40000" dist="23000" dir="5400000" rotWithShape="0">
+            <a:outerShdw blurRad="40000" dir="5400000" dist="23000" rotWithShape="0">
               <a:srgbClr val="000000">
                 <a:alpha val="35000"/>
               </a:srgbClr>
@@ -341,12 +341,12 @@
             <a:camera prst="orthographicFront">
               <a:rot lat="0" lon="0" rev="0"/>
             </a:camera>
-            <a:lightRig rig="threePt" dir="t">
+            <a:lightRig dir="t" rig="threePt">
               <a:rot lat="0" lon="0" rev="1200000"/>
             </a:lightRig>
           </a:scene3d>
           <a:sp3d>
-            <a:bevelT w="63500" h="25400"/>
+            <a:bevelT h="25400" w="63500"/>
           </a:sp3d>
         </a:effectStyle>
       </a:effectStyleLst>
@@ -377,7 +377,7 @@
             </a:gs>
           </a:gsLst>
           <a:path path="circle">
-            <a:fillToRect l="50000" t="-80000" r="50000" b="180000"/>
+            <a:fillToRect b="180000" l="50000" r="50000" t="-80000"/>
           </a:path>
         </a:gradFill>
         <a:gradFill rotWithShape="1">
@@ -396,7 +396,7 @@
             </a:gs>
           </a:gsLst>
           <a:path path="circle">
-            <a:fillToRect l="50000" t="50000" r="50000" b="50000"/>
+            <a:fillToRect b="50000" l="50000" r="50000" t="50000"/>
           </a:path>
         </a:gradFill>
       </a:bgFillStyleLst>
@@ -670,6 +670,6 @@
       </c>
     </row>
   </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageMargins bottom="1" footer="0.5" header="0.5" left="0.75" right="0.75" top="1"/>
 </worksheet>
 </file>
</xml_diff>